<commit_message>
Add sample syllabus files (Cambridge IGCSE, A Level, Lower Secondary) for syllabus parser
</commit_message>
<xml_diff>
--- a/public/syllabus/0893 Lower Secondary Science Learning Objectives Only.xlsx
+++ b/public/syllabus/0893 Lower Secondary Science Learning Objectives Only.xlsx
@@ -1,42 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cambridgeorg-my.sharepoint.com/personal/lesley_spence_cambridgeinternational_org/Documents/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\opencode\happySaturday\physics-command-center\public\syllabus\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="495" documentId="8_{9873FB6B-7CAC-4497-9035-B19AFDF7826F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{75AC04E4-A955-4789-862E-38101F1C287F}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B9CF8B9C-D113-4EE7-93F9-1941FC1D4EEE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2"/>
   </bookViews>
   <sheets>
-    <sheet name="Contents" sheetId="5" r:id="rId1"/>
-    <sheet name="Stage 7" sheetId="13" r:id="rId2"/>
-    <sheet name="Stage 8" sheetId="18" r:id="rId3"/>
-    <sheet name="Stage 9" sheetId="19" r:id="rId4"/>
+    <sheet name="Stage 7" sheetId="13" r:id="rId1"/>
+    <sheet name="Stage 8" sheetId="18" r:id="rId2"/>
+    <sheet name="Stage 9" sheetId="19" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Stage 7'!$C$2:$C$52</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Stage 8'!$C$2:$C$51</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Stage 9'!$C$2:$C$52</definedName>
-    <definedName name="_Hlk218499527" localSheetId="1">'Stage 7'!$C$35</definedName>
-    <definedName name="_Hlk218499527" localSheetId="2">'Stage 8'!$C$35</definedName>
-    <definedName name="_Hlk218499527" localSheetId="3">'Stage 9'!$C$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Stage 7'!$C$2:$C$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Stage 8'!$C$2:$C$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Stage 9'!$C$2:$C$52</definedName>
+    <definedName name="_Hlk218499527" localSheetId="0">'Stage 7'!$C$35</definedName>
+    <definedName name="_Hlk218499527" localSheetId="1">'Stage 8'!$C$35</definedName>
+    <definedName name="_Hlk218499527" localSheetId="2">'Stage 9'!$C$34</definedName>
     <definedName name="Four">#REF!</definedName>
-    <definedName name="One" localSheetId="1">'Stage 7'!$C$1</definedName>
-    <definedName name="One" localSheetId="2">'Stage 8'!$C$1</definedName>
-    <definedName name="One" localSheetId="3">'Stage 9'!$C$1</definedName>
+    <definedName name="One" localSheetId="0">'Stage 7'!$C$1</definedName>
+    <definedName name="One" localSheetId="1">'Stage 8'!$C$1</definedName>
+    <definedName name="One" localSheetId="2">'Stage 9'!$C$1</definedName>
     <definedName name="One">#REF!</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Contents!$A$1:$J$17</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Stage 7'!$C$1:$C$52</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'Stage 8'!$C$1:$C$51</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="3">'Stage 9'!$C$1:$C$52</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Stage 7'!$1:$2</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Stage 8'!$1:$2</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="3">'Stage 9'!$1:$2</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Stage 7'!$C$1:$C$52</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Stage 8'!$C$1:$C$51</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'Stage 9'!$C$1:$C$52</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Stage 7'!$1:$2</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Stage 8'!$1:$2</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Stage 9'!$1:$2</definedName>
     <definedName name="Three">#REF!</definedName>
     <definedName name="Two">#REF!</definedName>
   </definedNames>
@@ -59,45 +56,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="247">
-  <si>
-    <t>Contents</t>
-  </si>
-  <si>
-    <t>End of page</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">We are committed to making our documents accessible in accordance with the WCAG 2.2 Standard. We are always looking to improve the accessibility of our documents. If you find any problems or you think we are not meeting accessibility requirements, contact us at </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>info@cambridgeinternational.org</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> with the subject heading: Digital accessibility. If you need this document in a different format, contact us and supply your name, email address and requirements and we will respond within 15 working days.</t>
-    </r>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="239">
   <si>
     <t>End of spreadsheet</t>
   </si>
   <si>
-    <t xml:space="preserve">Stage 7 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stage 8 </t>
-  </si>
-  <si>
     <t>Stage 9</t>
   </si>
   <si>
@@ -105,17 +68,6 @@
   </si>
   <si>
     <t>Stage 8</t>
-  </si>
-  <si>
-    <t>This Cambridge Lower Secondary Science document contains worksheets for Stages 7 to 9 that list the learning objectives for the stage by strand.</t>
-  </si>
-  <si>
-    <t>Version 2.0, published February 2026.</t>
-  </si>
-  <si>
-    <t>© Cambridge University Press &amp; Assessment 2026
-Cambridge International Education is the name of our awarding body and a part of Cambridge University Press &amp; Assessment, which is a department of the University of Cambridge.
-Cambridge University Press &amp; Assessment retains the copyright on all its publications. Registered centres are permitted to copy material from this booklet for their own internal use. However, we cannot give permission to centres to copy any material that is acknowledged to a third party even for internal use within a centre.</t>
   </si>
   <si>
     <t>Science</t>
@@ -4642,8 +4594,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -4654,32 +4606,6 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="16"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -4707,14 +4633,6 @@
       <b/>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF088A08"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -4769,51 +4687,31 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -4824,9 +4722,17 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -4854,314 +4760,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>85726</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>9525</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>540386</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>138430</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="5" name="Text Box 11" descr="Cambridge Primary">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F067BC67-48AF-4107-BE9E-CD11C1846BF3}"/>
-            </a:ext>
-            <a:ext uri="{C183D7F6-B498-43B3-948B-1728B52AA6E4}">
-              <adec:decorative xmlns:adec="http://schemas.microsoft.com/office/drawing/2017/decorative" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="3133726" y="190500"/>
-          <a:ext cx="2893060" cy="309880"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr rot="0" spcFirstLastPara="0" vert="horz" wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720" numCol="1" spcCol="0" rtlCol="0" fromWordArt="0" anchor="t" anchorCtr="0" forceAA="0" compatLnSpc="1">
-          <a:prstTxWarp prst="textNoShape">
-            <a:avLst/>
-          </a:prstTxWarp>
-          <a:noAutofit/>
-        </a:bodyPr>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="r">
-            <a:lnSpc>
-              <a:spcPct val="110000"/>
-            </a:lnSpc>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-GB" sz="1100">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="MS Mincho" panose="02020609040205080304" pitchFamily="49" charset="-128"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>Cambridge Primary</a:t>
-          </a:r>
-          <a:endParaRPr lang="en-GB" sz="1100">
-            <a:solidFill>
-              <a:srgbClr val="0D0D0D"/>
-            </a:solidFill>
-            <a:effectLst/>
-            <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            <a:ea typeface="MS Mincho" panose="02020609040205080304" pitchFamily="49" charset="-128"/>
-            <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>447675</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>34925</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>455240</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
-    </xdr:to>
-    <xdr:cxnSp macro="">
-      <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="7" name="Straight Connector 6">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{56526A87-17C4-4E3B-AB90-59F829D3320A}"/>
-            </a:ext>
-            <a:ext uri="{C183D7F6-B498-43B3-948B-1728B52AA6E4}">
-              <adec:decorative xmlns:adec="http://schemas.microsoft.com/office/drawing/2017/decorative" val="1"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvCxnSpPr/>
-      </xdr:nvCxnSpPr>
-      <xdr:spPr>
-        <a:xfrm flipV="1">
-          <a:off x="4714875" y="215900"/>
-          <a:ext cx="1226765" cy="3175"/>
-        </a:xfrm>
-        <a:prstGeom prst="line">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:solidFill>
-            <a:schemeClr val="bg1"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="1">
-          <a:schemeClr val="accent6"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent6"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="accent6"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </xdr:style>
-    </xdr:cxnSp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>142875</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="8" name="TextBox 7" descr="Cambridge Primary Global Perspectives – learning objectives by Challenge, skill focus and topic">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C8E73866-35B3-4584-9549-452D307E9E8E}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="866775"/>
-          <a:ext cx="6381750" cy="781050"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="088A08"/>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-GB" sz="1800" b="1">
-              <a:solidFill>
-                <a:schemeClr val="bg1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>Cambridge Lower Secondary Science 0893</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-GB" sz="1800" b="1" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="bg1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>Learning objectives</a:t>
-          </a:r>
-          <a:endParaRPr lang="en-GB" sz="3200">
-            <a:solidFill>
-              <a:schemeClr val="bg1"/>
-            </a:solidFill>
-            <a:effectLst/>
-            <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>164465</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1" descr="Cambridge International Education logo">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{27F03638-4826-44F9-B403-C588429A6257}"/>
-            </a:ext>
-            <a:ext uri="{C183D7F6-B498-43B3-948B-1728B52AA6E4}">
-              <adec:decorative xmlns:adec="http://schemas.microsoft.com/office/drawing/2017/decorative" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill rotWithShape="1">
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:srcRect r="9986"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="6052344" cy="878840"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:extLst>
-          <a:ext uri="{53640926-AAD7-44D8-BBD7-CCE9431645EC}">
-            <a14:shadowObscured xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main"/>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5460,633 +5058,511 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{807CC567-E69F-4C41-8A69-964BBFA9DE47}">
-  <dimension ref="A1:J40"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.25" zeroHeight="1" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="10" width="9.140625" style="1" customWidth="1"/>
-    <col min="11" max="16384" width="9.140625" style="1" hidden="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2"/>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2"/>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2"/>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2"/>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2"/>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2"/>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2"/>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2"/>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2"/>
-    <row r="10" spans="1:10" ht="38.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="2" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" ht="58.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="B11" s="13"/>
-      <c r="C11" s="13"/>
-      <c r="D11" s="13"/>
-      <c r="E11" s="13"/>
-      <c r="F11" s="13"/>
-      <c r="G11" s="13"/>
-      <c r="H11" s="13"/>
-      <c r="I11" s="13"/>
-      <c r="J11" s="13"/>
-    </row>
-    <row r="12" spans="1:10" ht="24.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="10" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" ht="24.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="10" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" ht="24.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="10" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" ht="24.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" ht="129.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="B16" s="13"/>
-      <c r="C16" s="13"/>
-      <c r="D16" s="13"/>
-      <c r="E16" s="13"/>
-      <c r="F16" s="13"/>
-      <c r="G16" s="13"/>
-      <c r="H16" s="13"/>
-      <c r="I16" s="13"/>
-      <c r="J16" s="13"/>
-    </row>
-    <row r="17" spans="1:10" ht="96.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="14" t="s">
-        <v>2</v>
-      </c>
-      <c r="B17" s="14"/>
-      <c r="C17" s="14"/>
-      <c r="D17" s="14"/>
-      <c r="E17" s="14"/>
-      <c r="F17" s="14"/>
-      <c r="G17" s="14"/>
-      <c r="H17" s="14"/>
-      <c r="I17" s="14"/>
-      <c r="J17" s="14"/>
-    </row>
-    <row r="18" spans="1:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="3" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.2"/>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.2"/>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.2"/>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.2"/>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.2"/>
-    <row r="33" s="1" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="34" s="1" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="35" s="1" customFormat="1" hidden="1" x14ac:dyDescent="0.2"/>
-    <row r="36" s="1" customFormat="1" hidden="1" x14ac:dyDescent="0.2"/>
-    <row r="37" s="1" customFormat="1" hidden="1" x14ac:dyDescent="0.2"/>
-    <row r="38" s="1" customFormat="1" hidden="1" x14ac:dyDescent="0.2"/>
-    <row r="39" s="1" customFormat="1" hidden="1" x14ac:dyDescent="0.2"/>
-    <row r="40" s="1" customFormat="1" hidden="1" x14ac:dyDescent="0.2"/>
-  </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A11:J11"/>
-    <mergeCell ref="A16:J16"/>
-    <mergeCell ref="A17:J17"/>
-  </mergeCells>
-  <hyperlinks>
-    <hyperlink ref="A17:J17" r:id="rId1" display="We are committed to making our documents accessible in accordance with the WCAG 2.1 Standard. We are always looking to improve the accessibility of our documents. If you find any problems or you think we are not meeting accessibility requirements, contact us at info@cambridgeinternational.org with the subject heading: Digital accessibility. If you need this document in a different format, contact us and supply your name, email address and requirements and we will respond within 15 working days." xr:uid="{36B52643-A404-4072-9CD5-5DF41C78B696}"/>
-    <hyperlink ref="A12" location="'Stage 7'!A1" display="Stage 7 " xr:uid="{EB767944-F50C-4FAD-BF18-474CDB51F6EC}"/>
-    <hyperlink ref="A13:A14" location="'Stages 7 to 9'!A1" display="Stages 7 to 9" xr:uid="{AF3D822B-F1E8-41FC-AF58-0A21025CD816}"/>
-    <hyperlink ref="A13" location="'Stage 8'!A1" display="Stage 8 " xr:uid="{BCD2AEE9-3A06-4C92-A4B3-4F1E4157CB22}"/>
-    <hyperlink ref="A14" location="'Stage 9'!One" display="Stage 9" xr:uid="{F303A755-DFDA-4D6F-BCF3-D6FEFD1A896A}"/>
-  </hyperlinks>
-  <pageMargins left="0.70866141732283472" right="0.31496062992125984" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
-  <drawing r:id="rId3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{878D76A9-3E6F-4144-81CB-F398462FE64E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:Z185"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="20.100000000000001" customHeight="1" zeroHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="9.140625" style="4" hidden="1" customWidth="1"/>
-    <col min="3" max="3" width="255.5703125" style="4" customWidth="1"/>
-    <col min="4" max="26" width="0" style="4" hidden="1" customWidth="1"/>
-    <col min="27" max="16384" width="9.140625" style="4" hidden="1"/>
+    <col min="1" max="2" width="9.140625" style="13" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="255.5703125" style="13" customWidth="1"/>
+    <col min="4" max="26" width="0" style="13" hidden="1" customWidth="1"/>
+    <col min="27" max="16384" width="9.140625" style="13" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C1" s="7" t="s">
+    <row r="1" spans="1:3" s="11" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C1" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" s="11" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C2" s="4" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" s="11" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="12"/>
+      <c r="B3" s="12"/>
+      <c r="C3" s="6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" s="11" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="12"/>
+      <c r="B4" s="12"/>
+      <c r="C4" s="7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C5" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C6" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C7" s="7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C8" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C9" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C10" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C11" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C12" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C13" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C14" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C15" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C16" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C17" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C18" s="3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C19" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C20" s="3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C21" s="7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C22" s="3" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C23" s="3" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C24" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C25" s="3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C26" s="3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" s="11" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="12"/>
+      <c r="B27" s="12"/>
+      <c r="C27" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" s="11" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="12"/>
+      <c r="B28" s="12"/>
+      <c r="C28" s="7" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C29" s="3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C30" s="3" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C31" s="3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C32" s="3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C33" s="3" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C34" s="7" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:3" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C2" s="7" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="8"/>
-      <c r="B3" s="8"/>
-      <c r="C3" s="9" t="s">
+    <row r="35" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C35" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C36" s="3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C37" s="3" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C38" s="3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C39" s="7" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:3" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="8"/>
-      <c r="B4" s="8"/>
-      <c r="C4" s="11" t="s">
+    <row r="40" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C40" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C41" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" s="11" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="12"/>
+      <c r="B42" s="12"/>
+      <c r="C42" s="6" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C5" s="6" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C6" s="6" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C7" s="11" t="s">
+    <row r="43" spans="1:3" s="11" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="12"/>
+      <c r="B43" s="12"/>
+      <c r="C43" s="7" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C8" s="6" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C9" s="6" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C10" s="6" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C11" s="6" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C12" s="6" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C13" s="11" t="s">
+    <row r="44" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C44" s="3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C45" s="3" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C46" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C47" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C48" s="3" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="49" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C49" s="3" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="50" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C50" s="3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="51" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C51" s="7" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C14" s="6" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C15" s="6" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C16" s="6" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C17" s="6" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C18" s="6" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C19" s="6" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C20" s="6" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C21" s="11" t="s">
+    <row r="52" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C52" s="3" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="53" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C53" s="3" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="54" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C54" s="3" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="55" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C55" s="3" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="56" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C56" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="57" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C57" s="3" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="58" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C58" s="3" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="59" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C59" s="7" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C22" s="6" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C23" s="6" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C24" s="6" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C25" s="6" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C26" s="6" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="8"/>
-      <c r="B27" s="8"/>
-      <c r="C27" s="9" t="s">
+    <row r="60" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C60" s="3" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="61" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C61" s="3" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="62" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C62" s="3" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="63" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C63" s="3" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="64" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C64" s="6" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="28" spans="1:3" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="8"/>
-      <c r="B28" s="8"/>
-      <c r="C28" s="11" t="s">
+    <row r="65" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C65" s="7" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C29" s="6" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C30" s="6" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C31" s="6" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C32" s="6" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C33" s="6" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C34" s="11" t="s">
+    <row r="66" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C66" s="3" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="67" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C67" s="3" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="68" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C68" s="3" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="69" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C69" s="3" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="70" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C70" s="7" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="35" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C35" s="6" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C36" s="6" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C37" s="6" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C38" s="6" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C39" s="11" t="s">
+    <row r="71" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C71" s="3" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="72" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C72" s="3" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="73" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C73" s="7" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="40" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C40" s="6" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C41" s="6" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="8"/>
-      <c r="B42" s="8"/>
-      <c r="C42" s="9" t="s">
+    <row r="74" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C74" s="3" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="75" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C75" s="3" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="76" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C76" s="3" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="77" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C77" s="3" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="78" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C78" s="3" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="79" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C79" s="6" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="43" spans="1:3" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="8"/>
-      <c r="B43" s="8"/>
-      <c r="C43" s="11" t="s">
+    <row r="80" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C80" s="7" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="44" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C44" s="6" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C45" s="6" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C46" s="6" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C47" s="6" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C48" s="6" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="49" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C49" s="6" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="50" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C50" s="6" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="51" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C51" s="11" t="s">
+    <row r="81" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C81" s="3" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="82" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C82" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="83" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C83" s="3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="84" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C84" s="7" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="52" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C52" s="6" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="53" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C53" s="6" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="54" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C54" s="6" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="55" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C55" s="6" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="56" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C56" s="6" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="57" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C57" s="6" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="58" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C58" s="6" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="59" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C59" s="11" t="s">
+    <row r="85" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C85" s="3" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="86" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C86" s="7" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="60" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C60" s="6" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="61" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C61" s="6" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="62" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C62" s="6" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="63" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C63" s="6" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="64" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C64" s="9" t="s">
+    <row r="87" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C87" s="3" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="88" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C88" s="3" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="89" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C89" s="3" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="90" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C90" s="3" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="91" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C91" s="6" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="65" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C65" s="11" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="66" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C66" s="6" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="67" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C67" s="6" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="68" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C68" s="6" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="69" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C69" s="6" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="70" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C70" s="11" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="71" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C71" s="6" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="72" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C72" s="6" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="73" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C73" s="11" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="74" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C74" s="6" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="75" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C75" s="6" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="76" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C76" s="6" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="77" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C77" s="6" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="78" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C78" s="6" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="79" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C79" s="9" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="80" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C80" s="11" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="81" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C81" s="6" t="s">
+    <row r="92" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C92" s="3" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="82" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C82" s="6" t="s">
+    <row r="93" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C93" s="3" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="83" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C83" s="6" t="s">
+    <row r="94" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C94" s="3" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="84" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C84" s="11" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="85" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C85" s="6" t="s">
+    <row r="95" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C95" s="3" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="86" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C86" s="11" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="87" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C87" s="6" t="s">
+    <row r="96" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C96" s="3" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="88" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C88" s="6" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="89" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C89" s="6" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="90" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C90" s="6" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="91" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C91" s="9" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="92" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C92" s="6" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="93" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C93" s="6" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="94" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C94" s="6" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="95" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C95" s="6" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="96" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C96" s="6" t="s">
-        <v>106</v>
-      </c>
-    </row>
     <row r="97" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C97" s="6" t="s">
-        <v>3</v>
+      <c r="C97" s="3" t="s">
+        <v>0</v>
       </c>
     </row>
     <row r="98" spans="3:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -6186,502 +5662,502 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3F9F0BC-39BB-45B2-B77C-46EEEA288EDD}">
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:Z196"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="20.100000000000001" customHeight="1" zeroHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="9.140625" style="4" hidden="1" customWidth="1"/>
-    <col min="3" max="3" width="255.5703125" style="4" customWidth="1"/>
-    <col min="4" max="26" width="0" style="4" hidden="1" customWidth="1"/>
-    <col min="27" max="16384" width="9.140625" style="4" hidden="1"/>
+    <col min="1" max="2" width="9.140625" style="1" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="255.5703125" style="1" customWidth="1"/>
+    <col min="4" max="26" width="0" style="1" hidden="1" customWidth="1"/>
+    <col min="27" max="16384" width="9.140625" style="1" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C1" s="7" t="s">
+    <row r="1" spans="1:3" s="2" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C1" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" s="2" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C2" s="4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" s="2" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="5"/>
+      <c r="B3" s="5"/>
+      <c r="C3" s="6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" s="2" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="5"/>
+      <c r="B4" s="5"/>
+      <c r="C4" s="7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C5" s="8" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C6" s="8" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C7" s="8" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C8" s="7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C9" s="8" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C10" s="8" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C11" s="8" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C12" s="8" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C13" s="8" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C14" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C15" s="8" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C16" s="8" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C17" s="8" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C18" s="8" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C19" s="8" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C20" s="8" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C21" s="8" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C22" s="7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C23" s="8" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C24" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C25" s="8" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C26" s="8" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C27" s="8" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" s="2" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="5"/>
+      <c r="B28" s="5"/>
+      <c r="C28" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" s="2" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="5"/>
+      <c r="B29" s="5"/>
+      <c r="C29" s="7" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C30" s="9" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C31" s="9" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C32" s="9" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C33" s="9" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C34" s="7" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:3" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C2" s="7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="8"/>
-      <c r="B3" s="8"/>
-      <c r="C3" s="9" t="s">
+    <row r="35" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C35" s="9" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C36" s="9" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C37" s="9" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C38" s="9" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C39" s="9" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C40" s="7" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:3" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="8"/>
-      <c r="B4" s="8"/>
-      <c r="C4" s="11" t="s">
+    <row r="41" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C41" s="9" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C42" s="9" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C43" s="9" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" s="2" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="5"/>
+      <c r="B44" s="5"/>
+      <c r="C44" s="6" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C5" s="15" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C6" s="15" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C7" s="15" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C8" s="11" t="s">
+    <row r="45" spans="1:3" s="2" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="5"/>
+      <c r="B45" s="5"/>
+      <c r="C45" s="7" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C9" s="15" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C10" s="15" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C11" s="15" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C12" s="15" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C13" s="15" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C14" s="11" t="s">
+    <row r="46" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C46" s="9" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C47" s="9" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C48" s="9" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="49" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C49" s="9" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="50" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C50" s="7" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C15" s="15" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C16" s="15" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C17" s="15" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C18" s="15" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C19" s="15" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C20" s="15" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C21" s="15" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C22" s="11" t="s">
+    <row r="51" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C51" s="9" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="52" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C52" s="9" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="53" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C53" s="7" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C23" s="15" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C24" s="15" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C25" s="15" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C26" s="15" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C27" s="15" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="8"/>
-      <c r="B28" s="8"/>
-      <c r="C28" s="9" t="s">
+    <row r="54" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C54" s="9" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="55" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C55" s="9" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="56" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C56" s="9" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="57" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C57" s="9" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="58" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C58" s="9" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="59" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C59" s="9" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="60" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C60" s="6" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:3" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="8"/>
-      <c r="B29" s="8"/>
-      <c r="C29" s="11" t="s">
+    <row r="61" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C61" s="7" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="30" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C30" s="16" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C31" s="16" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C32" s="16" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C33" s="16" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C34" s="11" t="s">
+    <row r="62" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C62" s="9" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="63" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C63" s="9" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="64" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C64" s="9" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="65" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C65" s="9" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="66" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C66" s="9" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="67" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C67" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="68" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C68" s="9" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="69" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C69" s="7" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="35" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C35" s="16" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C36" s="16" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C37" s="16" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C38" s="16" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C39" s="16" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C40" s="11" t="s">
+    <row r="70" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C70" s="9" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="71" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C71" s="9" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="72" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C72" s="9" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="73" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C73" s="9" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="74" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C74" s="7" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="41" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C41" s="16" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C42" s="16" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C43" s="16" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="8"/>
-      <c r="B44" s="8"/>
-      <c r="C44" s="9" t="s">
+    <row r="75" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C75" s="9" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="76" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C76" s="9" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="77" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C77" s="9" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="78" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C78" s="6" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="45" spans="1:3" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="8"/>
-      <c r="B45" s="8"/>
-      <c r="C45" s="11" t="s">
+    <row r="79" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C79" s="7" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="46" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C46" s="16" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C47" s="16" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C48" s="16" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="49" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C49" s="16" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="50" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C50" s="11" t="s">
+    <row r="80" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C80" s="9" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="81" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C81" s="9" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="82" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C82" s="7" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="51" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C51" s="16" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="52" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C52" s="16" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="53" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C53" s="11" t="s">
+    <row r="83" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C83" s="9" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="84" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C84" s="9" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="85" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C85" s="9" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="86" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C86" s="7" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="54" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C54" s="16" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="55" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C55" s="16" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="56" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C56" s="16" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="57" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C57" s="16" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="58" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C58" s="16" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="59" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C59" s="16" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="60" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C60" s="9" t="s">
+    <row r="87" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C87" s="9" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="88" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C88" s="9" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="89" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C89" s="6" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="61" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C61" s="11" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="62" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C62" s="16" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="63" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C63" s="16" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="64" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C64" s="16" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="65" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C65" s="16" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="66" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C66" s="16" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="67" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C67" s="16" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="68" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C68" s="16" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="69" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C69" s="11" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="70" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C70" s="16" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="71" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C71" s="16" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="72" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C72" s="16" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="73" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C73" s="16" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="74" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C74" s="11" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="75" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C75" s="16" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="76" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C76" s="16" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="77" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C77" s="16" t="s">
+    <row r="90" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C90" s="8" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="78" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C78" s="9" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="79" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C79" s="11" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="80" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C80" s="16" t="s">
+    <row r="91" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C91" s="8" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="81" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C81" s="16" t="s">
+    <row r="92" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C92" s="8" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="82" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C82" s="11" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="83" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C83" s="16" t="s">
+    <row r="93" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C93" s="8" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="84" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C84" s="16" t="s">
+    <row r="94" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C94" s="8" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="85" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C85" s="16" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="86" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C86" s="11" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="87" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C87" s="16" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="88" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C88" s="16" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="89" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C89" s="9" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="90" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C90" s="15" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="91" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C91" s="15" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="92" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C92" s="15" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="93" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C93" s="15" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="94" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C94" s="15" t="s">
-        <v>176</v>
-      </c>
-    </row>
     <row r="95" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C95" s="6" t="s">
-        <v>3</v>
+      <c r="C95" s="3" t="s">
+        <v>0</v>
       </c>
     </row>
     <row r="96" spans="3:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -6794,502 +6270,502 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33E330AF-378B-4458-A51B-DAB21CC53579}">
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:Z193"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="20.100000000000001" customHeight="1" zeroHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="9.140625" style="4" hidden="1" customWidth="1"/>
-    <col min="3" max="3" width="255.5703125" style="4" customWidth="1"/>
-    <col min="4" max="26" width="0" style="4" hidden="1" customWidth="1"/>
-    <col min="27" max="16384" width="9.140625" style="4" hidden="1"/>
+    <col min="1" max="2" width="9.140625" style="1" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="255.5703125" style="1" customWidth="1"/>
+    <col min="4" max="26" width="0" style="1" hidden="1" customWidth="1"/>
+    <col min="27" max="16384" width="9.140625" style="1" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C1" s="7" t="s">
+    <row r="1" spans="1:3" s="2" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C1" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" s="2" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C2" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" s="2" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="5"/>
+      <c r="B3" s="5"/>
+      <c r="C3" s="6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" s="2" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="5"/>
+      <c r="B4" s="5"/>
+      <c r="C4" s="7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C5" s="3" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C6" s="3" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C7" s="3" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C8" s="7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C9" s="3" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C10" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C11" s="3" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C12" s="3" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C13" s="3" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C14" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C15" s="3" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C16" s="3" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C17" s="3" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C18" s="3" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C19" s="3" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C20" s="3" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C21" s="3" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C22" s="7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C23" s="3" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C24" s="3" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C25" s="3" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C26" s="3" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C27" s="3" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" s="2" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="5"/>
+      <c r="B28" s="5"/>
+      <c r="C28" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" s="2" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="5"/>
+      <c r="B29" s="5"/>
+      <c r="C29" s="7" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C30" s="3" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C31" s="3" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C32" s="3" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C33" s="7" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:3" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C2" s="7" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="8"/>
-      <c r="B3" s="8"/>
-      <c r="C3" s="9" t="s">
+    <row r="34" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C34" s="3" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C35" s="3" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C36" s="3" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C37" s="3" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C38" s="3" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C39" s="3" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C40" s="3" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C41" s="3" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C42" s="7" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:3" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="8"/>
-      <c r="B4" s="8"/>
-      <c r="C4" s="11" t="s">
+    <row r="43" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C43" s="3" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" s="2" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="5"/>
+      <c r="B44" s="5"/>
+      <c r="C44" s="6" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C5" s="6" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C6" s="6" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C7" s="6" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C8" s="11" t="s">
+    <row r="45" spans="1:3" s="2" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="5"/>
+      <c r="B45" s="5"/>
+      <c r="C45" s="7" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C9" s="6" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C10" s="6" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C11" s="6" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C12" s="6" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C13" s="6" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C14" s="11" t="s">
+    <row r="46" spans="1:3" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C46" s="8" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C47" s="3" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C48" s="3" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="49" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C49" s="3" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="50" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C50" s="3" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="51" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C51" s="7" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C15" s="6" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C16" s="6" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C17" s="6" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C18" s="6" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C19" s="6" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C20" s="6" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C21" s="6" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C22" s="11" t="s">
+    <row r="52" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C52" s="3" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="53" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C53" s="3" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="54" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C54" s="3" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="55" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C55" s="3" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="56" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C56" s="7" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C23" s="6" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C24" s="6" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C25" s="6" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C26" s="6" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C27" s="6" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="8"/>
-      <c r="B28" s="8"/>
-      <c r="C28" s="9" t="s">
+    <row r="57" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C57" s="3" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="58" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C58" s="3" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="59" spans="3:3" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C59" s="8" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="60" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C60" s="3" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="61" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C61" s="3" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="62" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C62" s="6" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:3" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="8"/>
-      <c r="B29" s="8"/>
-      <c r="C29" s="11" t="s">
+    <row r="63" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C63" s="7" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="30" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C30" s="6" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C31" s="6" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C32" s="6" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C33" s="11" t="s">
+    <row r="64" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C64" s="10" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="65" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C65" s="10" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="66" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C66" s="10" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="67" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C67" s="10" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="68" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C68" s="10" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="69" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C69" s="10" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="70" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C70" s="7" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="34" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C34" s="6" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C35" s="6" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C36" s="6" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C37" s="6" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C38" s="6" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C39" s="6" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C40" s="6" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C41" s="6" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C42" s="11" t="s">
+    <row r="71" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C71" s="10" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="72" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C72" s="10" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="73" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C73" s="7" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="43" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C43" s="6" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="8"/>
-      <c r="B44" s="8"/>
-      <c r="C44" s="9" t="s">
+    <row r="74" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C74" s="10" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="75" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C75" s="10" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="76" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C76" s="10" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="77" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C77" s="10" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="78" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C78" s="6" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="45" spans="1:3" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="8"/>
-      <c r="B45" s="8"/>
-      <c r="C45" s="11" t="s">
+    <row r="79" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C79" s="7" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="46" spans="1:3" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C46" s="15" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C47" s="6" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C48" s="6" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="49" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C49" s="6" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="50" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C50" s="6" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="51" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C51" s="11" t="s">
+    <row r="80" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C80" s="10" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="81" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C81" s="10" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="82" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C82" s="7" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="52" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C52" s="6" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="53" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C53" s="6" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="54" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C54" s="6" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="55" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C55" s="6" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="56" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C56" s="11" t="s">
+    <row r="83" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C83" s="10" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="84" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C84" s="10" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="85" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C85" s="7" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="57" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C57" s="6" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="58" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C58" s="6" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="59" spans="3:3" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C59" s="15" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="60" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C60" s="6" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="61" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C61" s="6" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="62" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C62" s="9" t="s">
+    <row r="86" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C86" s="10" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="87" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C87" s="10" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="88" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C88" s="10" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="89" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C89" s="6" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="63" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C63" s="11" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="64" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C64" s="17" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="65" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C65" s="17" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="66" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C66" s="17" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="67" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C67" s="17" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="68" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C68" s="17" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="69" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C69" s="17" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="70" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C70" s="11" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="71" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C71" s="17" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="72" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C72" s="17" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="73" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C73" s="11" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="74" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C74" s="17" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="75" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C75" s="17" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="76" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C76" s="17" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="77" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C77" s="17" t="s">
+    <row r="90" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C90" s="3" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="78" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C78" s="9" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="79" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C79" s="11" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="80" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C80" s="17" t="s">
+    <row r="91" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C91" s="3" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="81" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C81" s="17" t="s">
+    <row r="92" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C92" s="3" t="s">
         <v>236</v>
       </c>
     </row>
-    <row r="82" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C82" s="11" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="83" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C83" s="17" t="s">
+    <row r="93" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C93" s="3" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="84" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C84" s="17" t="s">
+    <row r="94" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C94" s="10" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="85" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C85" s="11" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="86" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C86" s="17" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="87" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C87" s="17" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="88" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C88" s="17" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="89" spans="3:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C89" s="9" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="90" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C90" s="6" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="91" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C91" s="6" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="92" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C92" s="6" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="93" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C93" s="6" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="94" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C94" s="17" t="s">
-        <v>246</v>
-      </c>
-    </row>
     <row r="95" spans="3:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C95" s="6" t="s">
-        <v>3</v>
+      <c r="C95" s="3" t="s">
+        <v>0</v>
       </c>
     </row>
     <row r="96" spans="3:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -7400,14 +6876,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="487a0a52-7d7c-4cd2-bd53-1415b73631cd">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b1020240-084a-446a-804d-5d41bf97331b" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -7640,15 +7114,44 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="487a0a52-7d7c-4cd2-bd53-1415b73631cd">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b1020240-084a-446a-804d-5d41bf97331b" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9104C013-2891-4A0D-9440-23CB53EF4BA7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BC27EAC5-9358-4932-BA17-95A37C299CB6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="487a0a52-7d7c-4cd2-bd53-1415b73631cd"/>
+    <ds:schemaRef ds:uri="b1020240-084a-446a-804d-5d41bf97331b"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{240CD857-B97F-4A5B-A377-3690BC53A864}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
@@ -7663,18 +7166,8 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BC27EAC5-9358-4932-BA17-95A37C299CB6}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9104C013-2891-4A0D-9440-23CB53EF4BA7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="487a0a52-7d7c-4cd2-bd53-1415b73631cd"/>
+    <ds:schemaRef ds:uri="b1020240-084a-446a-804d-5d41bf97331b"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>